<commit_message>
docs: update validation sheets - add phase2-5 check (36 items) and test (23 cases)
</commit_message>
<xml_diff>
--- a/ESTA_バリデーション完全版.xlsx
+++ b/ESTA_バリデーション完全版.xlsx
@@ -19,6 +19,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Step5 確認テスト" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Step6 実装チェック" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Step6 確認テスト" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="フェーズ2〜5チェック" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="フェーズ2〜5テスト" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Step1 実装チェック'!$A$1:$H$157</definedName>
@@ -41,7 +43,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,8 +56,12 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -70,6 +76,36 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A3A5C"/>
+        <bgColor rgb="001A3A5C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+        <bgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEEFF"/>
+        <bgColor rgb="00DDEEFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -91,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -106,6 +142,22 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -7847,6 +7899,2257 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>フェーズ</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>カテゴリ</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>チェック項目</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>チェック内容</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>実装状況</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>更新日</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>フェーズ2</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>カメラガイド</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>カメラモーダル表示</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>「📷 カメラで撮影」でカメラモーダルが全画面表示</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>フェーズ2</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>カメラガイド</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>人型シルエット</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>頭部正円＋肩ラインのシルエット描画（arc()のみ・ellipse禁止）</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>フェーズ2</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>カメラガイド</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>明るさ判定</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>輝度70未満→警告 / 70-220→OK / 220超→警告</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>フェーズ2</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>カメラガイド</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>顔位置判定</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>FaceDetector対応時：中央ズレ&gt;20%で「中央に合わせて」</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>フェーズ2</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>カメラガイド</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>顔サイズ判定</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>比率&lt;0.4→「近づいて」 / &gt;0.75→「離れて」</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>フェーズ2</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>カメラガイド</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>自動シャッタートグル</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>OFF(デフォルト)/ON切替ボタン</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>フェーズ2</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>カメラガイド</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>自動シャッター発火</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>ON時：全条件OK 0.5秒→ポップアップ→自動撮影</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>フェーズ2</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>カメラガイド</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>非対応フォールバック</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>FaceDetector非対応時は明るさのみで自動シャッター判定</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>フェーズ2</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>カメラガイド</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>EXIF回転補正</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>JPEG EXIFからorientation読取→Canvas描画時補正</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>フェーズ2</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>品質チェック</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>品質チェックUI</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>明るさ・解像度・形式の結果表示</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>フェーズ2</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>品質チェック</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>写真使用ボタン</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>NGなしの場合のみ「この写真を使用する」表示</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>フェーズ2</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>品質チェック</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>再撮影導線</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>「再撮影する」でカメラガイドに戻る</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>フェーズ3</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>QR転送</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>QRボタン</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>PC表示時のみ顔写真欄に「📱 スマホから送信」表示</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>フェーズ3</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>QR転送</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>PeerJS接続</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>PeerJS経由でPeerID生成→QRコード表示</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>フェーズ3</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>QR転送</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>5分タイムアウト</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>5分でQRグレーアウト・期限切れ表示</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>フェーズ3</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>QR転送</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>SP専用UI</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>?peer=XXXアクセスでフォーム非表示→専用UI</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>フェーズ3</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>QR転送</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>SP撮影→PC送信</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>カメラガイドで撮影→600×600処理→WebRTC転送</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>フェーズ3</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>QR転送</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>PC受信プレビュー</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>受信後PCにプレビュー表示→自動クローズ</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>フェーズ3</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>QR転送</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>PeerID1回限り</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>受信後peer.destroy()でセッション破棄</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>フェーズ3</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>QR転送</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>フォールバック</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>getUserMedia失敗→ネイティブカメラに自動切替</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>フェーズ4</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>品質担保</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>自動背景補正</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>顔領域外→白方向35%ブレンド＋影リフト</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>フェーズ4</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>品質担保</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>顔コーナーガイド</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>FaceDetector時にコーナーブラケット白枠表示</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>フェーズ4</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>品質担保</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>品質スコア0-100</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>明るさ25pt+顔サイズ25pt+顔位置25pt+背景25pt</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>フェーズ4</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>品質担保</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>スコア判定</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>90以上:✅ / 60-89:⚠️ / 60未満:❌</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G25" s="9" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>フェーズ4</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>品質担保</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>60未満で使用不可</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>スコア60未満→「この写真を使用する」ボタン非表示</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>フェーズ4</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>分析ログ</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>イベント記録</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>camera_open/capture/accepted/retakenをlocalStorageに保存</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>フェーズ4</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>分析ログ</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>デバッグパネル</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>?debug=1で統計パネル表示（起動/採用/平均スコア）</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>フェーズ5</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>パスポートOCR</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t>OCR自動起動</t>
+        </is>
+      </c>
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>アップロード完了後に自動でTesseract.js MRZ解析</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G29" s="10" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>フェーズ5</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>パスポートOCR</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="inlineStr">
+        <is>
+          <t>MRZ自動入力</t>
+        </is>
+      </c>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>姓・名・番号・生年月日・有効期限・性別を自動入力</t>
+        </is>
+      </c>
+      <c r="F30" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G30" s="10" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>フェーズ5</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>パスポートOCR</t>
+        </is>
+      </c>
+      <c r="D31" s="10" t="inlineStr">
+        <is>
+          <t>読取状況表示</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>「読み取り中」→「✅X項目自動入力」または「❌失敗」</t>
+        </is>
+      </c>
+      <c r="F31" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G31" s="10" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>フェーズ5</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>パスポートOCR</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>再読み取りボタン</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>完了後に「🔄 再読み取り」ボタン表示</t>
+        </is>
+      </c>
+      <c r="F32" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G32" s="10" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>フェーズ5</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>autofill</t>
+        </is>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
+        <is>
+          <t>autocomplete属性</t>
+        </is>
+      </c>
+      <c r="E33" s="10" t="inlineStr">
+        <is>
+          <t>主要フィールドにautocomplete属性を付与</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G33" s="10" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>フェーズ5</t>
+        </is>
+      </c>
+      <c r="C34" s="10" t="inlineStr">
+        <is>
+          <t>入力履歴</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>自動保存</t>
+        </is>
+      </c>
+      <c r="E34" s="10" t="inlineStr">
+        <is>
+          <t>nextStep()時にlocalStorageへ自動保存</t>
+        </is>
+      </c>
+      <c r="F34" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G34" s="10" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>フェーズ5</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>入力履歴</t>
+        </is>
+      </c>
+      <c r="D35" s="10" t="inlineStr">
+        <is>
+          <t>復元バー</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="inlineStr">
+        <is>
+          <t>次回アクセス時に復元バーを10秒表示</t>
+        </is>
+      </c>
+      <c r="F35" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G35" s="10" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>フェーズ5</t>
+        </is>
+      </c>
+      <c r="C36" s="10" t="inlineStr">
+        <is>
+          <t>入力履歴</t>
+        </is>
+      </c>
+      <c r="D36" s="10" t="inlineStr">
+        <is>
+          <t>7日自動削除</t>
+        </is>
+      </c>
+      <c r="E36" s="10" t="inlineStr">
+        <is>
+          <t>7日超のドラフトを自動削除</t>
+        </is>
+      </c>
+      <c r="F36" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G36" s="10" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>フェーズ5</t>
+        </is>
+      </c>
+      <c r="C37" s="10" t="inlineStr">
+        <is>
+          <t>メールサジェスト</t>
+        </is>
+      </c>
+      <c r="D37" s="10" t="inlineStr">
+        <is>
+          <t>ドメイン候補</t>
+        </is>
+      </c>
+      <c r="E37" s="10" t="inlineStr">
+        <is>
+          <t>@入力後にドメイン候補を最大4件表示</t>
+        </is>
+      </c>
+      <c r="F37" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G37" s="10" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>テストID</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>フェーズ</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>カテゴリ</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>操作</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>期待結果</t>
+        </is>
+      </c>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t>結果</t>
+        </is>
+      </c>
+      <c r="G1" s="11" t="inlineStr">
+        <is>
+          <t>備考</t>
+        </is>
+      </c>
+      <c r="H1" s="11" t="inlineStr">
+        <is>
+          <t>更新日</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>P2-001</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>フェーズ2</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>カメラガイド</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>スマホで「📷 カメラで撮影」タップ</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>カメラモーダルが全画面表示・人型ガイド描画</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr"/>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>P2-002</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>フェーズ2</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>明るさ判定</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>暗い場所でカメラを向ける</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>「明るい場所で撮影してください」表示</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>P2-003</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>フェーズ2</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>自動シャッター</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>「🔴 自動 OFF」タップ</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>「🟢 自動 ON」に変わる</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>P2-004</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>フェーズ2</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>自動撮影</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>自動ON・全条件0.5秒クリア</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>「自動撮影します！」→自動撮影</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>P2-005</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>フェーズ2</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>品質チェック</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>撮影後</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>品質チェック結果が表示される</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>P2-006</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>フェーズ2</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>再撮影</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>「再撮影する」タップ</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>カメラガイドに戻る</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>P3-001</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>フェーズ3</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>QRボタン</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>PC表示で顔写真欄を確認</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>「📱 スマホから送信（QR）」ボタン表示</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr"/>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>P3-002</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>フェーズ3</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>QR生成</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>「📱 スマホから送信」クリック</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>QRコード＋カウントダウンバー表示</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr"/>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>P3-003</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>フェーズ3</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>SP専用UI</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>QRのURLをスマホで開く</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>フォーム非表示→「顔写真をPCに送信」UI表示</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr"/>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>P3-004</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>フェーズ3</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>タイムアウト</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>QR表示後5分放置</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>QRグレーアウト・期限切れ表示</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr"/>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>P3-005</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>フェーズ3</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>SP→PC転送</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>SP側で撮影して送信</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>PC側に写真がプレビュー表示</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr"/>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>P4-001</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>フェーズ4</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>品質スコア</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>撮影後の品質チェック画面を確認</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>0-100スコア＋ゲージバー表示</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="inlineStr"/>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>P4-002</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>フェーズ4</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>スコア90以上</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>十分な明るさ・正面・適切サイズで撮影</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>✅高品質・「使用する」ボタン表示</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr"/>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>P4-003</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>フェーズ4</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>スコア60未満</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>暗い・顔小さい等のNG条件で撮影</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>❌再撮影推奨・「使用する」ボタン非表示</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr"/>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>P4-004</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>フェーズ4</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>デバッグ</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>?debug=1でアクセス</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>撮影統計パネルが下部に表示</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr"/>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>P5-001</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>フェーズ5</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>OCR自動起動</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>パスポート画像をアップロード</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>「🔍 パスポートを読み取り中」が自動表示</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="inlineStr"/>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>P5-002</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>フェーズ5</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>OCR自動入力</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>日本パスポートをアップロード</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>姓・名・番号・生年月日・有効期限・性別が自動入力</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="inlineStr"/>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>P5-003</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>フェーズ5</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>OCR失敗</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>ぼやけた画像をアップロード</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>「❌ MRZ読取失敗」＋再読み取りボタン表示</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="inlineStr"/>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>P5-004</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>フェーズ5</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>履歴保存</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>Step1入力後にStep2へ</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>localStorageに保存される</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr"/>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>P5-005</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>フェーズ5</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>履歴復元</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>保存後にリロード</t>
+        </is>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>「📋 前回の入力内容があります」バー表示</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G21" s="10" t="inlineStr"/>
+      <c r="H21" s="10" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>P5-006</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>フェーズ5</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>復元実行</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>「復元する」クリック</t>
+        </is>
+      </c>
+      <c r="E22" s="10" t="inlineStr">
+        <is>
+          <t>前回値が各フィールドに復元</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G22" s="10" t="inlineStr"/>
+      <c r="H22" s="10" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>P5-007</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>フェーズ5</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>メールサジェスト</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>emailで「test@」入力</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="inlineStr">
+        <is>
+          <t>gmail.com等の候補が最大4件表示</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="inlineStr"/>
+      <c r="H23" s="10" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>P5-008</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>フェーズ5</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>サジェスト選択</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>候補をクリック</t>
+        </is>
+      </c>
+      <c r="E24" s="10" t="inlineStr">
+        <is>
+          <t>メールアドレスが補完される</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G24" s="10" t="inlineStr"/>
+      <c r="H24" s="10" t="inlineStr">
+        <is>
+          <t>2026/04/06</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
docs: integrate phase2-5 items into Step1 sheets of complete validation file
</commit_message>
<xml_diff>
--- a/ESTA_バリデーション完全版.xlsx
+++ b/ESTA_バリデーション完全版.xlsx
@@ -19,8 +19,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Step5 確認テスト" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Step6 実装チェック" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Step6 確認テスト" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="フェーズ2〜5チェック" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="フェーズ2〜5テスト" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Step1 実装チェック'!$A$1:$H$157</definedName>
@@ -43,7 +41,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,8 +58,13 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -108,6 +111,18 @@
         <bgColor rgb="00DDEEFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002D5F8A"/>
+        <bgColor rgb="002D5F8A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F4FD"/>
+        <bgColor rgb="00E8F4FD"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -127,7 +142,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -158,6 +173,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -523,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H157"/>
+  <dimension ref="A1:H192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6577,6 +6598,1284 @@
         </is>
       </c>
       <c r="H157" s="2" t="n"/>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr"/>
+      <c r="B158" t="inlineStr"/>
+      <c r="C158" t="inlineStr"/>
+      <c r="D158" t="inlineStr"/>
+      <c r="E158" t="inlineStr"/>
+      <c r="F158" t="inlineStr"/>
+      <c r="G158" t="inlineStr"/>
+      <c r="H158" t="inlineStr"/>
+    </row>
+    <row r="159" ht="20" customHeight="1">
+      <c r="A159" s="12" t="inlineStr">
+        <is>
+          <t>【フェーズ2〜5追加】カメラ機能 / QR転送 / OCR自動入力 / 自動補完</t>
+        </is>
+      </c>
+      <c r="B159" s="12" t="inlineStr"/>
+      <c r="C159" s="12" t="inlineStr"/>
+      <c r="D159" s="12" t="inlineStr"/>
+      <c r="E159" s="12" t="inlineStr"/>
+      <c r="F159" s="12" t="inlineStr"/>
+      <c r="G159" s="12" t="inlineStr"/>
+      <c r="H159" s="12" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="13" t="inlineStr">
+        <is>
+          <t>顔写真アップロード</t>
+        </is>
+      </c>
+      <c r="B160" s="13" t="inlineStr">
+        <is>
+          <t>カメラモーダル</t>
+        </is>
+      </c>
+      <c r="C160" s="13" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="D160" s="13" t="inlineStr">
+        <is>
+          <t>カメラモーダル表示</t>
+        </is>
+      </c>
+      <c r="E160" s="13" t="inlineStr">
+        <is>
+          <t>「📷 カメラで撮影」タップで全画面カメラモーダルが開く</t>
+        </is>
+      </c>
+      <c r="F160" s="13" t="inlineStr">
+        <is>
+          <t>openCameraModal()実装</t>
+        </is>
+      </c>
+      <c r="G160" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H160" s="13" t="n"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="13" t="inlineStr">
+        <is>
+          <t>顔写真アップロード</t>
+        </is>
+      </c>
+      <c r="B161" s="13" t="inlineStr">
+        <is>
+          <t>カメラガイド</t>
+        </is>
+      </c>
+      <c r="C161" s="13" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="D161" s="13" t="inlineStr">
+        <is>
+          <t>人型シルエット描画</t>
+        </is>
+      </c>
+      <c r="E161" s="13" t="inlineStr">
+        <is>
+          <t>Canvas上に頭部正円(arc()のみ)+肩ベジェ曲線を描画</t>
+        </is>
+      </c>
+      <c r="F161" s="13" t="inlineStr">
+        <is>
+          <t>drawHumanGuide()実装</t>
+        </is>
+      </c>
+      <c r="G161" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H161" s="13" t="n"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="13" t="inlineStr">
+        <is>
+          <t>顔写真アップロード</t>
+        </is>
+      </c>
+      <c r="B162" s="13" t="inlineStr">
+        <is>
+          <t>カメラガイド</t>
+        </is>
+      </c>
+      <c r="C162" s="13" t="inlineStr">
+        <is>
+          <t>P03</t>
+        </is>
+      </c>
+      <c r="D162" s="13" t="inlineStr">
+        <is>
+          <t>明るさ判定リアルタイム</t>
+        </is>
+      </c>
+      <c r="E162" s="13" t="inlineStr">
+        <is>
+          <t>平均輝度70未満→警告 / 70-220→OK / 220超→警告</t>
+        </is>
+      </c>
+      <c r="F162" s="13" t="inlineStr">
+        <is>
+          <t>calcBrightness()実装</t>
+        </is>
+      </c>
+      <c r="G162" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H162" s="13" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="13" t="inlineStr">
+        <is>
+          <t>顔写真アップロード</t>
+        </is>
+      </c>
+      <c r="B163" s="13" t="inlineStr">
+        <is>
+          <t>カメラガイド</t>
+        </is>
+      </c>
+      <c r="C163" s="13" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="D163" s="13" t="inlineStr">
+        <is>
+          <t>顔位置判定(FaceDetector)</t>
+        </is>
+      </c>
+      <c r="E163" s="13" t="inlineStr">
+        <is>
+          <t>中央ズレ&gt;20%で「中央に合わせてください」表示</t>
+        </is>
+      </c>
+      <c r="F163" s="13" t="inlineStr">
+        <is>
+          <t>FaceDetector.detect()使用</t>
+        </is>
+      </c>
+      <c r="G163" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H163" s="13" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="13" t="inlineStr">
+        <is>
+          <t>顔写真アップロード</t>
+        </is>
+      </c>
+      <c r="B164" s="13" t="inlineStr">
+        <is>
+          <t>カメラガイド</t>
+        </is>
+      </c>
+      <c r="C164" s="13" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="D164" s="13" t="inlineStr">
+        <is>
+          <t>顔サイズ判定</t>
+        </is>
+      </c>
+      <c r="E164" s="13" t="inlineStr">
+        <is>
+          <t>比率&lt;0.4→「近づいて」 / &gt;0.75→「離れて」</t>
+        </is>
+      </c>
+      <c r="F164" s="13" t="inlineStr">
+        <is>
+          <t>FaceDetector.boundingBox使用</t>
+        </is>
+      </c>
+      <c r="G164" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H164" s="13" t="n"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="13" t="inlineStr">
+        <is>
+          <t>顔写真アップロード</t>
+        </is>
+      </c>
+      <c r="B165" s="13" t="inlineStr">
+        <is>
+          <t>自動シャッター</t>
+        </is>
+      </c>
+      <c r="C165" s="13" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="D165" s="13" t="inlineStr">
+        <is>
+          <t>自動シャッタートグル</t>
+        </is>
+      </c>
+      <c r="E165" s="13" t="inlineStr">
+        <is>
+          <t>OFF(デフォルト)/ONをボタンで切り替え</t>
+        </is>
+      </c>
+      <c r="F165" s="13" t="inlineStr">
+        <is>
+          <t>camAutoShutterOn フラグ</t>
+        </is>
+      </c>
+      <c r="G165" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H165" s="13" t="n"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="13" t="inlineStr">
+        <is>
+          <t>顔写真アップロード</t>
+        </is>
+      </c>
+      <c r="B166" s="13" t="inlineStr">
+        <is>
+          <t>自動シャッター</t>
+        </is>
+      </c>
+      <c r="C166" s="13" t="inlineStr">
+        <is>
+          <t>P07</t>
+        </is>
+      </c>
+      <c r="D166" s="13" t="inlineStr">
+        <is>
+          <t>自動シャッター発火</t>
+        </is>
+      </c>
+      <c r="E166" s="13" t="inlineStr">
+        <is>
+          <t>ON時：全条件OK 0.5秒継続→ポップアップ→自動撮影</t>
+        </is>
+      </c>
+      <c r="F166" s="13" t="inlineStr">
+        <is>
+          <t>camOkStart タイマー</t>
+        </is>
+      </c>
+      <c r="G166" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H166" s="13" t="n"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="13" t="inlineStr">
+        <is>
+          <t>顔写真アップロード</t>
+        </is>
+      </c>
+      <c r="B167" s="13" t="inlineStr">
+        <is>
+          <t>自動シャッター</t>
+        </is>
+      </c>
+      <c r="C167" s="13" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="D167" s="13" t="inlineStr">
+        <is>
+          <t>非対応ブラウザフォールバック</t>
+        </is>
+      </c>
+      <c r="E167" s="13" t="inlineStr">
+        <is>
+          <t>FaceDetector非対応時は明るさのみで自動シャッター判定</t>
+        </is>
+      </c>
+      <c r="F167" s="13" t="inlineStr">
+        <is>
+          <t>camFaceDetector===null 分岐</t>
+        </is>
+      </c>
+      <c r="G167" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H167" s="13" t="n"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="13" t="inlineStr">
+        <is>
+          <t>顔写真アップロード</t>
+        </is>
+      </c>
+      <c r="B168" s="13" t="inlineStr">
+        <is>
+          <t>カメラ撮影</t>
+        </is>
+      </c>
+      <c r="C168" s="13" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="D168" s="13" t="inlineStr">
+        <is>
+          <t>EXIF回転補正</t>
+        </is>
+      </c>
+      <c r="E168" s="13" t="inlineStr">
+        <is>
+          <t>JPEG EXIFのorientation読取→Canvas描画時に自動回転補正</t>
+        </is>
+      </c>
+      <c r="F168" s="13" t="inlineStr">
+        <is>
+          <t>EXIF解析ロジック実装</t>
+        </is>
+      </c>
+      <c r="G168" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H168" s="13" t="n"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="13" t="inlineStr">
+        <is>
+          <t>顔写真アップロード</t>
+        </is>
+      </c>
+      <c r="B169" s="13" t="inlineStr">
+        <is>
+          <t>品質スコア</t>
+        </is>
+      </c>
+      <c r="C169" s="13" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="D169" s="13" t="inlineStr">
+        <is>
+          <t>品質スコア算出(0-100点)</t>
+        </is>
+      </c>
+      <c r="E169" s="13" t="inlineStr">
+        <is>
+          <t>明るさ25pt+顔サイズ25pt+顔位置25pt+背景均一性25ptの合計</t>
+        </is>
+      </c>
+      <c r="F169" s="13" t="inlineStr">
+        <is>
+          <t>calcQualityScore()実装</t>
+        </is>
+      </c>
+      <c r="G169" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H169" s="13" t="n"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="13" t="inlineStr">
+        <is>
+          <t>顔写真アップロード</t>
+        </is>
+      </c>
+      <c r="B170" s="13" t="inlineStr">
+        <is>
+          <t>品質スコア</t>
+        </is>
+      </c>
+      <c r="C170" s="13" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="D170" s="13" t="inlineStr">
+        <is>
+          <t>スコア判定ライン</t>
+        </is>
+      </c>
+      <c r="E170" s="13" t="inlineStr">
+        <is>
+          <t>90以上:✅高品質 / 60-89:⚠️使用可 / 60未満:❌再撮影推奨</t>
+        </is>
+      </c>
+      <c r="F170" s="13" t="inlineStr">
+        <is>
+          <t>showQualityCheck()分岐</t>
+        </is>
+      </c>
+      <c r="G170" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H170" s="13" t="n"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="13" t="inlineStr">
+        <is>
+          <t>顔写真アップロード</t>
+        </is>
+      </c>
+      <c r="B171" s="13" t="inlineStr">
+        <is>
+          <t>品質スコア</t>
+        </is>
+      </c>
+      <c r="C171" s="13" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="D171" s="13" t="inlineStr">
+        <is>
+          <t>60未満で使用ボタン非表示</t>
+        </is>
+      </c>
+      <c r="E171" s="13" t="inlineStr">
+        <is>
+          <t>スコア60未満の場合「この写真を使用する」ボタンを非表示</t>
+        </is>
+      </c>
+      <c r="F171" s="13" t="inlineStr">
+        <is>
+          <t>score&lt;60判定</t>
+        </is>
+      </c>
+      <c r="G171" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H171" s="13" t="n"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="13" t="inlineStr">
+        <is>
+          <t>顔写真アップロード</t>
+        </is>
+      </c>
+      <c r="B172" s="13" t="inlineStr">
+        <is>
+          <t>背景補正</t>
+        </is>
+      </c>
+      <c r="C172" s="13" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="D172" s="13" t="inlineStr">
+        <is>
+          <t>自動背景補正</t>
+        </is>
+      </c>
+      <c r="E172" s="13" t="inlineStr">
+        <is>
+          <t>顔領域外ピクセルを白方向35%ブレンド＋影リフト処理</t>
+        </is>
+      </c>
+      <c r="F172" s="13" t="inlineStr">
+        <is>
+          <t>applyBgCorrection()実装</t>
+        </is>
+      </c>
+      <c r="G172" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H172" s="13" t="n"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="13" t="inlineStr">
+        <is>
+          <t>顔写真アップロード</t>
+        </is>
+      </c>
+      <c r="B173" s="13" t="inlineStr">
+        <is>
+          <t>顔ガイド枠</t>
+        </is>
+      </c>
+      <c r="C173" s="13" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="D173" s="13" t="inlineStr">
+        <is>
+          <t>顔コーナーブラケット表示</t>
+        </is>
+      </c>
+      <c r="E173" s="13" t="inlineStr">
+        <is>
+          <t>FaceDetector検出時にコーナーブラケット白枠を描画</t>
+        </is>
+      </c>
+      <c r="F173" s="13" t="inlineStr">
+        <is>
+          <t>drawFeedback()実装</t>
+        </is>
+      </c>
+      <c r="G173" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H173" s="13" t="n"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="13" t="inlineStr">
+        <is>
+          <t>顔写真アップロード</t>
+        </is>
+      </c>
+      <c r="B174" s="13" t="inlineStr">
+        <is>
+          <t>QR転送</t>
+        </is>
+      </c>
+      <c r="C174" s="13" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="D174" s="13" t="inlineStr">
+        <is>
+          <t>QRボタン(PC限定表示)</t>
+        </is>
+      </c>
+      <c r="E174" s="13" t="inlineStr">
+        <is>
+          <t>PC表示時のみ「📱 スマホから送信（QR）」ボタンを表示</t>
+        </is>
+      </c>
+      <c r="F174" s="13" t="inlineStr">
+        <is>
+          <t>upload-btns-pc クラス</t>
+        </is>
+      </c>
+      <c r="G174" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H174" s="13" t="n"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="13" t="inlineStr">
+        <is>
+          <t>顔写真アップロード</t>
+        </is>
+      </c>
+      <c r="B175" s="13" t="inlineStr">
+        <is>
+          <t>QR転送</t>
+        </is>
+      </c>
+      <c r="C175" s="13" t="inlineStr">
+        <is>
+          <t>P16</t>
+        </is>
+      </c>
+      <c r="D175" s="13" t="inlineStr">
+        <is>
+          <t>PeerJS接続・QR生成</t>
+        </is>
+      </c>
+      <c r="E175" s="13" t="inlineStr">
+        <is>
+          <t>ボタン押下でPeerID生成→QRコード(qrserver.com)表示</t>
+        </is>
+      </c>
+      <c r="F175" s="13" t="inlineStr">
+        <is>
+          <t>openQRTransfer()実装</t>
+        </is>
+      </c>
+      <c r="G175" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H175" s="13" t="n"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="13" t="inlineStr">
+        <is>
+          <t>顔写真アップロード</t>
+        </is>
+      </c>
+      <c r="B176" s="13" t="inlineStr">
+        <is>
+          <t>QR転送</t>
+        </is>
+      </c>
+      <c r="C176" s="13" t="inlineStr">
+        <is>
+          <t>P17</t>
+        </is>
+      </c>
+      <c r="D176" s="13" t="inlineStr">
+        <is>
+          <t>5分タイムアウト</t>
+        </is>
+      </c>
+      <c r="E176" s="13" t="inlineStr">
+        <is>
+          <t>5分経過でQRグレーアウト・「期限切れ」表示</t>
+        </is>
+      </c>
+      <c r="F176" s="13" t="inlineStr">
+        <is>
+          <t>PEER_TIMEOUT_MS=300000</t>
+        </is>
+      </c>
+      <c r="G176" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H176" s="13" t="n"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="13" t="inlineStr">
+        <is>
+          <t>顔写真アップロード</t>
+        </is>
+      </c>
+      <c r="B177" s="13" t="inlineStr">
+        <is>
+          <t>QR転送</t>
+        </is>
+      </c>
+      <c r="C177" s="13" t="inlineStr">
+        <is>
+          <t>P18</t>
+        </is>
+      </c>
+      <c r="D177" s="13" t="inlineStr">
+        <is>
+          <t>SP専用UI</t>
+        </is>
+      </c>
+      <c r="E177" s="13" t="inlineStr">
+        <is>
+          <t>?peer=XXXアクセスでフォーム非表示→専用UI(#spReceiverUI)表示</t>
+        </is>
+      </c>
+      <c r="F177" s="13" t="inlineStr">
+        <is>
+          <t>URLパラメータ検出</t>
+        </is>
+      </c>
+      <c r="G177" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H177" s="13" t="n"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="13" t="inlineStr">
+        <is>
+          <t>顔写真アップロード</t>
+        </is>
+      </c>
+      <c r="B178" s="13" t="inlineStr">
+        <is>
+          <t>QR転送</t>
+        </is>
+      </c>
+      <c r="C178" s="13" t="inlineStr">
+        <is>
+          <t>P19</t>
+        </is>
+      </c>
+      <c r="D178" s="13" t="inlineStr">
+        <is>
+          <t>SP撮影→PC WebRTC転送</t>
+        </is>
+      </c>
+      <c r="E178" s="13" t="inlineStr">
+        <is>
+          <t>SP撮影→600×600処理→ArrayBufferでPC側にWebRTC転送</t>
+        </is>
+      </c>
+      <c r="F178" s="13" t="inlineStr">
+        <is>
+          <t>PeerJS DataChannel使用</t>
+        </is>
+      </c>
+      <c r="G178" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H178" s="13" t="n"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="13" t="inlineStr">
+        <is>
+          <t>顔写真アップロード</t>
+        </is>
+      </c>
+      <c r="B179" s="13" t="inlineStr">
+        <is>
+          <t>QR転送</t>
+        </is>
+      </c>
+      <c r="C179" s="13" t="inlineStr">
+        <is>
+          <t>P20</t>
+        </is>
+      </c>
+      <c r="D179" s="13" t="inlineStr">
+        <is>
+          <t>PC受信プレビュー・自動クローズ</t>
+        </is>
+      </c>
+      <c r="E179" s="13" t="inlineStr">
+        <is>
+          <t>受信後PCのQRモーダルにプレビュー→3秒後自動クローズ</t>
+        </is>
+      </c>
+      <c r="F179" s="13" t="inlineStr">
+        <is>
+          <t>ondata イベント処理</t>
+        </is>
+      </c>
+      <c r="G179" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H179" s="13" t="n"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="13" t="inlineStr">
+        <is>
+          <t>顔写真アップロード</t>
+        </is>
+      </c>
+      <c r="B180" s="13" t="inlineStr">
+        <is>
+          <t>QR転送</t>
+        </is>
+      </c>
+      <c r="C180" s="13" t="inlineStr">
+        <is>
+          <t>P21</t>
+        </is>
+      </c>
+      <c r="D180" s="13" t="inlineStr">
+        <is>
+          <t>PeerID1回限り</t>
+        </is>
+      </c>
+      <c r="E180" s="13" t="inlineStr">
+        <is>
+          <t>写真受信後にpeer.destroy()でセッション破棄</t>
+        </is>
+      </c>
+      <c r="F180" s="13" t="inlineStr">
+        <is>
+          <t>peer.destroy()実装</t>
+        </is>
+      </c>
+      <c r="G180" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H180" s="13" t="n"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="13" t="inlineStr">
+        <is>
+          <t>顔写真アップロード</t>
+        </is>
+      </c>
+      <c r="B181" s="13" t="inlineStr">
+        <is>
+          <t>QR転送</t>
+        </is>
+      </c>
+      <c r="C181" s="13" t="inlineStr">
+        <is>
+          <t>P22</t>
+        </is>
+      </c>
+      <c r="D181" s="13" t="inlineStr">
+        <is>
+          <t>getUserMediaフォールバック</t>
+        </is>
+      </c>
+      <c r="E181" s="13" t="inlineStr">
+        <is>
+          <t>getUserMedia失敗時はネイティブ&lt;input capture&gt;に自動切替</t>
+        </is>
+      </c>
+      <c r="F181" s="13" t="inlineStr">
+        <is>
+          <t>try/catch フォールバック</t>
+        </is>
+      </c>
+      <c r="G181" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H181" s="13" t="n"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="13" t="inlineStr">
+        <is>
+          <t>顔写真アップロード</t>
+        </is>
+      </c>
+      <c r="B182" s="13" t="inlineStr">
+        <is>
+          <t>分析ログ</t>
+        </is>
+      </c>
+      <c r="C182" s="13" t="inlineStr">
+        <is>
+          <t>P23</t>
+        </is>
+      </c>
+      <c r="D182" s="13" t="inlineStr">
+        <is>
+          <t>撮影イベント記録</t>
+        </is>
+      </c>
+      <c r="E182" s="13" t="inlineStr">
+        <is>
+          <t>camera_open/capture/photo_accepted/photo_retakenをlocalStorageに保存</t>
+        </is>
+      </c>
+      <c r="F182" s="13" t="inlineStr">
+        <is>
+          <t>logEvent()実装</t>
+        </is>
+      </c>
+      <c r="G182" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H182" s="13" t="n"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="13" t="inlineStr">
+        <is>
+          <t>顔写真アップロード</t>
+        </is>
+      </c>
+      <c r="B183" s="13" t="inlineStr">
+        <is>
+          <t>分析ログ</t>
+        </is>
+      </c>
+      <c r="C183" s="13" t="inlineStr">
+        <is>
+          <t>P24</t>
+        </is>
+      </c>
+      <c r="D183" s="13" t="inlineStr">
+        <is>
+          <t>デバッグパネル</t>
+        </is>
+      </c>
+      <c r="E183" s="13" t="inlineStr">
+        <is>
+          <t>?debug=1アクセスで起動回数・採用率・平均スコアのパネル表示</t>
+        </is>
+      </c>
+      <c r="F183" s="13" t="inlineStr">
+        <is>
+          <t>showDebugPanel()実装</t>
+        </is>
+      </c>
+      <c r="G183" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H183" s="13" t="n"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="13" t="inlineStr">
+        <is>
+          <t>パスポートアップロード</t>
+        </is>
+      </c>
+      <c r="B184" s="13" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C184" s="13" t="inlineStr">
+        <is>
+          <t>P25</t>
+        </is>
+      </c>
+      <c r="D184" s="13" t="inlineStr">
+        <is>
+          <t>OCR自動起動</t>
+        </is>
+      </c>
+      <c r="E184" s="13" t="inlineStr">
+        <is>
+          <t>パスポートアップロード完了後に自動でTesseract.js MRZ解析を起動</t>
+        </is>
+      </c>
+      <c r="F184" s="13" t="inlineStr">
+        <is>
+          <t>handleUpload()→runPassportOCR()</t>
+        </is>
+      </c>
+      <c r="G184" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H184" s="13" t="n"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="13" t="inlineStr">
+        <is>
+          <t>パスポートアップロード</t>
+        </is>
+      </c>
+      <c r="B185" s="13" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C185" s="13" t="inlineStr">
+        <is>
+          <t>P26</t>
+        </is>
+      </c>
+      <c r="D185" s="13" t="inlineStr">
+        <is>
+          <t>MRZ解析・自動入力</t>
+        </is>
+      </c>
+      <c r="E185" s="13" t="inlineStr">
+        <is>
+          <t>MRZ読取成功時に姓・名・番号・生年月日・有効期限・性別を自動入力</t>
+        </is>
+      </c>
+      <c r="F185" s="13" t="inlineStr">
+        <is>
+          <t>parseMRZ()→fillFromOCR()</t>
+        </is>
+      </c>
+      <c r="G185" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H185" s="13" t="n"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="13" t="inlineStr">
+        <is>
+          <t>パスポートアップロード</t>
+        </is>
+      </c>
+      <c r="B186" s="13" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C186" s="13" t="inlineStr">
+        <is>
+          <t>P27</t>
+        </is>
+      </c>
+      <c r="D186" s="13" t="inlineStr">
+        <is>
+          <t>読取状況表示</t>
+        </is>
+      </c>
+      <c r="E186" s="13" t="inlineStr">
+        <is>
+          <t>「🔍 読み取り中」→「✅X項目自動入力」または「❌失敗」を表示</t>
+        </is>
+      </c>
+      <c r="F186" s="13" t="inlineStr">
+        <is>
+          <t>showOCRStatus()実装</t>
+        </is>
+      </c>
+      <c r="G186" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H186" s="13" t="n"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="13" t="inlineStr">
+        <is>
+          <t>パスポートアップロード</t>
+        </is>
+      </c>
+      <c r="B187" s="13" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C187" s="13" t="inlineStr">
+        <is>
+          <t>P28</t>
+        </is>
+      </c>
+      <c r="D187" s="13" t="inlineStr">
+        <is>
+          <t>再読み取りボタン</t>
+        </is>
+      </c>
+      <c r="E187" s="13" t="inlineStr">
+        <is>
+          <t>完了後に「🔄 再読み取り」ボタンを表示し手動再実行が可能</t>
+        </is>
+      </c>
+      <c r="F187" s="13" t="inlineStr">
+        <is>
+          <t>ocrBtn 表示制御</t>
+        </is>
+      </c>
+      <c r="G187" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H187" s="13" t="n"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="13" t="inlineStr">
+        <is>
+          <t>全体</t>
+        </is>
+      </c>
+      <c r="B188" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C188" s="13" t="inlineStr">
+        <is>
+          <t>P29</t>
+        </is>
+      </c>
+      <c r="D188" s="13" t="inlineStr">
+        <is>
+          <t>autofill属性付与</t>
+        </is>
+      </c>
+      <c r="E188" s="13" t="inlineStr">
+        <is>
+          <t>surname/givenName/email/phoneNumber/street/zipCodeにautocomplete属性</t>
+        </is>
+      </c>
+      <c r="F188" s="13" t="inlineStr">
+        <is>
+          <t>JS動的付与</t>
+        </is>
+      </c>
+      <c r="G188" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H188" s="13" t="n"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="13" t="inlineStr">
+        <is>
+          <t>全体</t>
+        </is>
+      </c>
+      <c r="B189" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C189" s="13" t="inlineStr">
+        <is>
+          <t>P30</t>
+        </is>
+      </c>
+      <c r="D189" s="13" t="inlineStr">
+        <is>
+          <t>入力履歴自動保存</t>
+        </is>
+      </c>
+      <c r="E189" s="13" t="inlineStr">
+        <is>
+          <t>nextStep()実行時にフォームデータをlocalStorageに自動保存</t>
+        </is>
+      </c>
+      <c r="F189" s="13" t="inlineStr">
+        <is>
+          <t>saveFormDraft()実装</t>
+        </is>
+      </c>
+      <c r="G189" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H189" s="13" t="n"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="13" t="inlineStr">
+        <is>
+          <t>全体</t>
+        </is>
+      </c>
+      <c r="B190" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C190" s="13" t="inlineStr">
+        <is>
+          <t>P31</t>
+        </is>
+      </c>
+      <c r="D190" s="13" t="inlineStr">
+        <is>
+          <t>入力履歴復元バー</t>
+        </is>
+      </c>
+      <c r="E190" s="13" t="inlineStr">
+        <is>
+          <t>次回アクセス時に「📋 前回の入力内容があります」バーを10秒表示</t>
+        </is>
+      </c>
+      <c r="F190" s="13" t="inlineStr">
+        <is>
+          <t>DOMContentLoaded検出</t>
+        </is>
+      </c>
+      <c r="G190" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H190" s="13" t="n"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="13" t="inlineStr">
+        <is>
+          <t>全体</t>
+        </is>
+      </c>
+      <c r="B191" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C191" s="13" t="inlineStr">
+        <is>
+          <t>P32</t>
+        </is>
+      </c>
+      <c r="D191" s="13" t="inlineStr">
+        <is>
+          <t>7日自動削除</t>
+        </is>
+      </c>
+      <c r="E191" s="13" t="inlineStr">
+        <is>
+          <t>保存から7日以上経過したドラフトを自動削除</t>
+        </is>
+      </c>
+      <c r="F191" s="13" t="inlineStr">
+        <is>
+          <t>Date.now()差分判定</t>
+        </is>
+      </c>
+      <c r="G191" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H191" s="13" t="n"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="13" t="inlineStr">
+        <is>
+          <t>申請者情報</t>
+        </is>
+      </c>
+      <c r="B192" s="13" t="inlineStr">
+        <is>
+          <t>メールアドレス</t>
+        </is>
+      </c>
+      <c r="C192" s="13" t="inlineStr">
+        <is>
+          <t>P33</t>
+        </is>
+      </c>
+      <c r="D192" s="13" t="inlineStr">
+        <is>
+          <t>メールドメインサジェスト</t>
+        </is>
+      </c>
+      <c r="E192" s="13" t="inlineStr">
+        <is>
+          <t>@入力後にgmail.com/yahoo.co.jp等の候補を最大4件表示</t>
+        </is>
+      </c>
+      <c r="F192" s="13" t="inlineStr">
+        <is>
+          <t>input イベントリスナー</t>
+        </is>
+      </c>
+      <c r="G192" s="13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H192" s="13" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H157"/>
@@ -7899,2264 +9198,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G37"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="B1" s="6" t="inlineStr">
-        <is>
-          <t>フェーズ</t>
-        </is>
-      </c>
-      <c r="C1" s="6" t="inlineStr">
-        <is>
-          <t>カテゴリ</t>
-        </is>
-      </c>
-      <c r="D1" s="6" t="inlineStr">
-        <is>
-          <t>チェック項目</t>
-        </is>
-      </c>
-      <c r="E1" s="6" t="inlineStr">
-        <is>
-          <t>チェック内容</t>
-        </is>
-      </c>
-      <c r="F1" s="6" t="inlineStr">
-        <is>
-          <t>実装状況</t>
-        </is>
-      </c>
-      <c r="G1" s="6" t="inlineStr">
-        <is>
-          <t>更新日</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>フェーズ2</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>カメラガイド</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>カメラモーダル表示</t>
-        </is>
-      </c>
-      <c r="E2" s="7" t="inlineStr">
-        <is>
-          <t>「📷 カメラで撮影」でカメラモーダルが全画面表示</t>
-        </is>
-      </c>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G2" s="7" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>フェーズ2</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>カメラガイド</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>人型シルエット</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>頭部正円＋肩ラインのシルエット描画（arc()のみ・ellipse禁止）</t>
-        </is>
-      </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G3" s="7" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>フェーズ2</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>カメラガイド</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>明るさ判定</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>輝度70未満→警告 / 70-220→OK / 220超→警告</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G4" s="7" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>フェーズ2</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>カメラガイド</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>顔位置判定</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>FaceDetector対応時：中央ズレ&gt;20%で「中央に合わせて」</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>フェーズ2</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>カメラガイド</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>顔サイズ判定</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>比率&lt;0.4→「近づいて」 / &gt;0.75→「離れて」</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>フェーズ2</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>カメラガイド</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>自動シャッタートグル</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>OFF(デフォルト)/ON切替ボタン</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>フェーズ2</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>カメラガイド</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>自動シャッター発火</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>ON時：全条件OK 0.5秒→ポップアップ→自動撮影</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G8" s="7" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>フェーズ2</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>カメラガイド</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>非対応フォールバック</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>FaceDetector非対応時は明るさのみで自動シャッター判定</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G9" s="7" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>フェーズ2</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>カメラガイド</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>EXIF回転補正</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>JPEG EXIFからorientation読取→Canvas描画時補正</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>フェーズ2</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>品質チェック</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>品質チェックUI</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>明るさ・解像度・形式の結果表示</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G11" s="7" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>フェーズ2</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>品質チェック</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>写真使用ボタン</t>
-        </is>
-      </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>NGなしの場合のみ「この写真を使用する」表示</t>
-        </is>
-      </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G12" s="7" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>フェーズ2</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>品質チェック</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>再撮影導線</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>「再撮影する」でカメラガイドに戻る</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G13" s="7" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="8" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>フェーズ3</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>QR転送</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>QRボタン</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>PC表示時のみ顔写真欄に「📱 スマホから送信」表示</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>フェーズ3</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>QR転送</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>PeerJS接続</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>PeerJS経由でPeerID生成→QRコード表示</t>
-        </is>
-      </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G15" s="8" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="8" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>フェーズ3</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>QR転送</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>5分タイムアウト</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>5分でQRグレーアウト・期限切れ表示</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G16" s="8" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>フェーズ3</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>QR転送</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>SP専用UI</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>?peer=XXXアクセスでフォーム非表示→専用UI</t>
-        </is>
-      </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G17" s="8" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="8" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>フェーズ3</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>QR転送</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>SP撮影→PC送信</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="inlineStr">
-        <is>
-          <t>カメラガイドで撮影→600×600処理→WebRTC転送</t>
-        </is>
-      </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G18" s="8" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="8" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>フェーズ3</t>
-        </is>
-      </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>QR転送</t>
-        </is>
-      </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>PC受信プレビュー</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="inlineStr">
-        <is>
-          <t>受信後PCにプレビュー表示→自動クローズ</t>
-        </is>
-      </c>
-      <c r="F19" s="8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G19" s="8" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>フェーズ3</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>QR転送</t>
-        </is>
-      </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>PeerID1回限り</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>受信後peer.destroy()でセッション破棄</t>
-        </is>
-      </c>
-      <c r="F20" s="8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G20" s="8" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>フェーズ3</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>QR転送</t>
-        </is>
-      </c>
-      <c r="D21" s="8" t="inlineStr">
-        <is>
-          <t>フォールバック</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>getUserMedia失敗→ネイティブカメラに自動切替</t>
-        </is>
-      </c>
-      <c r="F21" s="8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G21" s="8" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="9" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>フェーズ4</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>品質担保</t>
-        </is>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>自動背景補正</t>
-        </is>
-      </c>
-      <c r="E22" s="9" t="inlineStr">
-        <is>
-          <t>顔領域外→白方向35%ブレンド＋影リフト</t>
-        </is>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G22" s="9" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="9" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>フェーズ4</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>品質担保</t>
-        </is>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>顔コーナーガイド</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>FaceDetector時にコーナーブラケット白枠表示</t>
-        </is>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G23" s="9" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="9" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>フェーズ4</t>
-        </is>
-      </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>品質担保</t>
-        </is>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>品質スコア0-100</t>
-        </is>
-      </c>
-      <c r="E24" s="9" t="inlineStr">
-        <is>
-          <t>明るさ25pt+顔サイズ25pt+顔位置25pt+背景25pt</t>
-        </is>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G24" s="9" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="9" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>フェーズ4</t>
-        </is>
-      </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>品質担保</t>
-        </is>
-      </c>
-      <c r="D25" s="9" t="inlineStr">
-        <is>
-          <t>スコア判定</t>
-        </is>
-      </c>
-      <c r="E25" s="9" t="inlineStr">
-        <is>
-          <t>90以上:✅ / 60-89:⚠️ / 60未満:❌</t>
-        </is>
-      </c>
-      <c r="F25" s="9" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G25" s="9" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="9" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>フェーズ4</t>
-        </is>
-      </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>品質担保</t>
-        </is>
-      </c>
-      <c r="D26" s="9" t="inlineStr">
-        <is>
-          <t>60未満で使用不可</t>
-        </is>
-      </c>
-      <c r="E26" s="9" t="inlineStr">
-        <is>
-          <t>スコア60未満→「この写真を使用する」ボタン非表示</t>
-        </is>
-      </c>
-      <c r="F26" s="9" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G26" s="9" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="9" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>フェーズ4</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>分析ログ</t>
-        </is>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
-        <is>
-          <t>イベント記録</t>
-        </is>
-      </c>
-      <c r="E27" s="9" t="inlineStr">
-        <is>
-          <t>camera_open/capture/accepted/retakenをlocalStorageに保存</t>
-        </is>
-      </c>
-      <c r="F27" s="9" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G27" s="9" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="9" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>フェーズ4</t>
-        </is>
-      </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>分析ログ</t>
-        </is>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
-        <is>
-          <t>デバッグパネル</t>
-        </is>
-      </c>
-      <c r="E28" s="9" t="inlineStr">
-        <is>
-          <t>?debug=1で統計パネル表示（起動/採用/平均スコア）</t>
-        </is>
-      </c>
-      <c r="F28" s="9" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G28" s="9" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="10" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" s="10" t="inlineStr">
-        <is>
-          <t>フェーズ5</t>
-        </is>
-      </c>
-      <c r="C29" s="10" t="inlineStr">
-        <is>
-          <t>パスポートOCR</t>
-        </is>
-      </c>
-      <c r="D29" s="10" t="inlineStr">
-        <is>
-          <t>OCR自動起動</t>
-        </is>
-      </c>
-      <c r="E29" s="10" t="inlineStr">
-        <is>
-          <t>アップロード完了後に自動でTesseract.js MRZ解析</t>
-        </is>
-      </c>
-      <c r="F29" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G29" s="10" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="10" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" s="10" t="inlineStr">
-        <is>
-          <t>フェーズ5</t>
-        </is>
-      </c>
-      <c r="C30" s="10" t="inlineStr">
-        <is>
-          <t>パスポートOCR</t>
-        </is>
-      </c>
-      <c r="D30" s="10" t="inlineStr">
-        <is>
-          <t>MRZ自動入力</t>
-        </is>
-      </c>
-      <c r="E30" s="10" t="inlineStr">
-        <is>
-          <t>姓・名・番号・生年月日・有効期限・性別を自動入力</t>
-        </is>
-      </c>
-      <c r="F30" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G30" s="10" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="10" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" s="10" t="inlineStr">
-        <is>
-          <t>フェーズ5</t>
-        </is>
-      </c>
-      <c r="C31" s="10" t="inlineStr">
-        <is>
-          <t>パスポートOCR</t>
-        </is>
-      </c>
-      <c r="D31" s="10" t="inlineStr">
-        <is>
-          <t>読取状況表示</t>
-        </is>
-      </c>
-      <c r="E31" s="10" t="inlineStr">
-        <is>
-          <t>「読み取り中」→「✅X項目自動入力」または「❌失敗」</t>
-        </is>
-      </c>
-      <c r="F31" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G31" s="10" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="10" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" s="10" t="inlineStr">
-        <is>
-          <t>フェーズ5</t>
-        </is>
-      </c>
-      <c r="C32" s="10" t="inlineStr">
-        <is>
-          <t>パスポートOCR</t>
-        </is>
-      </c>
-      <c r="D32" s="10" t="inlineStr">
-        <is>
-          <t>再読み取りボタン</t>
-        </is>
-      </c>
-      <c r="E32" s="10" t="inlineStr">
-        <is>
-          <t>完了後に「🔄 再読み取り」ボタン表示</t>
-        </is>
-      </c>
-      <c r="F32" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G32" s="10" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="10" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" s="10" t="inlineStr">
-        <is>
-          <t>フェーズ5</t>
-        </is>
-      </c>
-      <c r="C33" s="10" t="inlineStr">
-        <is>
-          <t>autofill</t>
-        </is>
-      </c>
-      <c r="D33" s="10" t="inlineStr">
-        <is>
-          <t>autocomplete属性</t>
-        </is>
-      </c>
-      <c r="E33" s="10" t="inlineStr">
-        <is>
-          <t>主要フィールドにautocomplete属性を付与</t>
-        </is>
-      </c>
-      <c r="F33" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G33" s="10" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="10" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" s="10" t="inlineStr">
-        <is>
-          <t>フェーズ5</t>
-        </is>
-      </c>
-      <c r="C34" s="10" t="inlineStr">
-        <is>
-          <t>入力履歴</t>
-        </is>
-      </c>
-      <c r="D34" s="10" t="inlineStr">
-        <is>
-          <t>自動保存</t>
-        </is>
-      </c>
-      <c r="E34" s="10" t="inlineStr">
-        <is>
-          <t>nextStep()時にlocalStorageへ自動保存</t>
-        </is>
-      </c>
-      <c r="F34" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G34" s="10" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="10" t="n">
-        <v>34</v>
-      </c>
-      <c r="B35" s="10" t="inlineStr">
-        <is>
-          <t>フェーズ5</t>
-        </is>
-      </c>
-      <c r="C35" s="10" t="inlineStr">
-        <is>
-          <t>入力履歴</t>
-        </is>
-      </c>
-      <c r="D35" s="10" t="inlineStr">
-        <is>
-          <t>復元バー</t>
-        </is>
-      </c>
-      <c r="E35" s="10" t="inlineStr">
-        <is>
-          <t>次回アクセス時に復元バーを10秒表示</t>
-        </is>
-      </c>
-      <c r="F35" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G35" s="10" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="10" t="n">
-        <v>35</v>
-      </c>
-      <c r="B36" s="10" t="inlineStr">
-        <is>
-          <t>フェーズ5</t>
-        </is>
-      </c>
-      <c r="C36" s="10" t="inlineStr">
-        <is>
-          <t>入力履歴</t>
-        </is>
-      </c>
-      <c r="D36" s="10" t="inlineStr">
-        <is>
-          <t>7日自動削除</t>
-        </is>
-      </c>
-      <c r="E36" s="10" t="inlineStr">
-        <is>
-          <t>7日超のドラフトを自動削除</t>
-        </is>
-      </c>
-      <c r="F36" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G36" s="10" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="10" t="n">
-        <v>36</v>
-      </c>
-      <c r="B37" s="10" t="inlineStr">
-        <is>
-          <t>フェーズ5</t>
-        </is>
-      </c>
-      <c r="C37" s="10" t="inlineStr">
-        <is>
-          <t>メールサジェスト</t>
-        </is>
-      </c>
-      <c r="D37" s="10" t="inlineStr">
-        <is>
-          <t>ドメイン候補</t>
-        </is>
-      </c>
-      <c r="E37" s="10" t="inlineStr">
-        <is>
-          <t>@入力後にドメイン候補を最大4件表示</t>
-        </is>
-      </c>
-      <c r="F37" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G37" s="10" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H24"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="11" t="inlineStr">
-        <is>
-          <t>テストID</t>
-        </is>
-      </c>
-      <c r="B1" s="11" t="inlineStr">
-        <is>
-          <t>フェーズ</t>
-        </is>
-      </c>
-      <c r="C1" s="11" t="inlineStr">
-        <is>
-          <t>カテゴリ</t>
-        </is>
-      </c>
-      <c r="D1" s="11" t="inlineStr">
-        <is>
-          <t>操作</t>
-        </is>
-      </c>
-      <c r="E1" s="11" t="inlineStr">
-        <is>
-          <t>期待結果</t>
-        </is>
-      </c>
-      <c r="F1" s="11" t="inlineStr">
-        <is>
-          <t>結果</t>
-        </is>
-      </c>
-      <c r="G1" s="11" t="inlineStr">
-        <is>
-          <t>備考</t>
-        </is>
-      </c>
-      <c r="H1" s="11" t="inlineStr">
-        <is>
-          <t>更新日</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>P2-001</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>フェーズ2</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>カメラガイド</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>スマホで「📷 カメラで撮影」タップ</t>
-        </is>
-      </c>
-      <c r="E2" s="7" t="inlineStr">
-        <is>
-          <t>カメラモーダルが全画面表示・人型ガイド描画</t>
-        </is>
-      </c>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G2" s="7" t="inlineStr"/>
-      <c r="H2" s="7" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>P2-002</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>フェーズ2</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>明るさ判定</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>暗い場所でカメラを向ける</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>「明るい場所で撮影してください」表示</t>
-        </is>
-      </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="7" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>P2-003</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>フェーズ2</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>自動シャッター</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>「🔴 自動 OFF」タップ</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>「🟢 自動 ON」に変わる</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>P2-004</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>フェーズ2</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>自動撮影</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>自動ON・全条件0.5秒クリア</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>「自動撮影します！」→自動撮影</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>P2-005</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>フェーズ2</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>品質チェック</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>撮影後</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>品質チェック結果が表示される</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>P2-006</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>フェーズ2</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>再撮影</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>「再撮影する」タップ</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>カメラガイドに戻る</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>P3-001</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>フェーズ3</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>QRボタン</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>PC表示で顔写真欄を確認</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>「📱 スマホから送信（QR）」ボタン表示</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G8" s="8" t="inlineStr"/>
-      <c r="H8" s="8" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>P3-002</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>フェーズ3</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>QR生成</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>「📱 スマホから送信」クリック</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>QRコード＋カウントダウンバー表示</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G9" s="8" t="inlineStr"/>
-      <c r="H9" s="8" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>P3-003</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>フェーズ3</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>SP専用UI</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>QRのURLをスマホで開く</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>フォーム非表示→「顔写真をPCに送信」UI表示</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G10" s="8" t="inlineStr"/>
-      <c r="H10" s="8" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>P3-004</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>フェーズ3</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>タイムアウト</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>QR表示後5分放置</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>QRグレーアウト・期限切れ表示</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G11" s="8" t="inlineStr"/>
-      <c r="H11" s="8" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>P3-005</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>フェーズ3</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>SP→PC転送</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>SP側で撮影して送信</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>PC側に写真がプレビュー表示</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G12" s="8" t="inlineStr"/>
-      <c r="H12" s="8" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>P4-001</t>
-        </is>
-      </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>フェーズ4</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>品質スコア</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>撮影後の品質チェック画面を確認</t>
-        </is>
-      </c>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t>0-100スコア＋ゲージバー表示</t>
-        </is>
-      </c>
-      <c r="F13" s="9" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G13" s="9" t="inlineStr"/>
-      <c r="H13" s="9" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>P4-002</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>フェーズ4</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>スコア90以上</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>十分な明るさ・正面・適切サイズで撮影</t>
-        </is>
-      </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>✅高品質・「使用する」ボタン表示</t>
-        </is>
-      </c>
-      <c r="F14" s="9" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G14" s="9" t="inlineStr"/>
-      <c r="H14" s="9" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>P4-003</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>フェーズ4</t>
-        </is>
-      </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>スコア60未満</t>
-        </is>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>暗い・顔小さい等のNG条件で撮影</t>
-        </is>
-      </c>
-      <c r="E15" s="9" t="inlineStr">
-        <is>
-          <t>❌再撮影推奨・「使用する」ボタン非表示</t>
-        </is>
-      </c>
-      <c r="F15" s="9" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G15" s="9" t="inlineStr"/>
-      <c r="H15" s="9" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>P4-004</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>フェーズ4</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>デバッグ</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>?debug=1でアクセス</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t>撮影統計パネルが下部に表示</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G16" s="9" t="inlineStr"/>
-      <c r="H16" s="9" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>P5-001</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>フェーズ5</t>
-        </is>
-      </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>OCR自動起動</t>
-        </is>
-      </c>
-      <c r="D17" s="10" t="inlineStr">
-        <is>
-          <t>パスポート画像をアップロード</t>
-        </is>
-      </c>
-      <c r="E17" s="10" t="inlineStr">
-        <is>
-          <t>「🔍 パスポートを読み取り中」が自動表示</t>
-        </is>
-      </c>
-      <c r="F17" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G17" s="10" t="inlineStr"/>
-      <c r="H17" s="10" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>P5-002</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>フェーズ5</t>
-        </is>
-      </c>
-      <c r="C18" s="10" t="inlineStr">
-        <is>
-          <t>OCR自動入力</t>
-        </is>
-      </c>
-      <c r="D18" s="10" t="inlineStr">
-        <is>
-          <t>日本パスポートをアップロード</t>
-        </is>
-      </c>
-      <c r="E18" s="10" t="inlineStr">
-        <is>
-          <t>姓・名・番号・生年月日・有効期限・性別が自動入力</t>
-        </is>
-      </c>
-      <c r="F18" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G18" s="10" t="inlineStr"/>
-      <c r="H18" s="10" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t>P5-003</t>
-        </is>
-      </c>
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t>フェーズ5</t>
-        </is>
-      </c>
-      <c r="C19" s="10" t="inlineStr">
-        <is>
-          <t>OCR失敗</t>
-        </is>
-      </c>
-      <c r="D19" s="10" t="inlineStr">
-        <is>
-          <t>ぼやけた画像をアップロード</t>
-        </is>
-      </c>
-      <c r="E19" s="10" t="inlineStr">
-        <is>
-          <t>「❌ MRZ読取失敗」＋再読み取りボタン表示</t>
-        </is>
-      </c>
-      <c r="F19" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G19" s="10" t="inlineStr"/>
-      <c r="H19" s="10" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="10" t="inlineStr">
-        <is>
-          <t>P5-004</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>フェーズ5</t>
-        </is>
-      </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>履歴保存</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>Step1入力後にStep2へ</t>
-        </is>
-      </c>
-      <c r="E20" s="10" t="inlineStr">
-        <is>
-          <t>localStorageに保存される</t>
-        </is>
-      </c>
-      <c r="F20" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G20" s="10" t="inlineStr"/>
-      <c r="H20" s="10" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>P5-005</t>
-        </is>
-      </c>
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t>フェーズ5</t>
-        </is>
-      </c>
-      <c r="C21" s="10" t="inlineStr">
-        <is>
-          <t>履歴復元</t>
-        </is>
-      </c>
-      <c r="D21" s="10" t="inlineStr">
-        <is>
-          <t>保存後にリロード</t>
-        </is>
-      </c>
-      <c r="E21" s="10" t="inlineStr">
-        <is>
-          <t>「📋 前回の入力内容があります」バー表示</t>
-        </is>
-      </c>
-      <c r="F21" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G21" s="10" t="inlineStr"/>
-      <c r="H21" s="10" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="10" t="inlineStr">
-        <is>
-          <t>P5-006</t>
-        </is>
-      </c>
-      <c r="B22" s="10" t="inlineStr">
-        <is>
-          <t>フェーズ5</t>
-        </is>
-      </c>
-      <c r="C22" s="10" t="inlineStr">
-        <is>
-          <t>復元実行</t>
-        </is>
-      </c>
-      <c r="D22" s="10" t="inlineStr">
-        <is>
-          <t>「復元する」クリック</t>
-        </is>
-      </c>
-      <c r="E22" s="10" t="inlineStr">
-        <is>
-          <t>前回値が各フィールドに復元</t>
-        </is>
-      </c>
-      <c r="F22" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G22" s="10" t="inlineStr"/>
-      <c r="H22" s="10" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="10" t="inlineStr">
-        <is>
-          <t>P5-007</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t>フェーズ5</t>
-        </is>
-      </c>
-      <c r="C23" s="10" t="inlineStr">
-        <is>
-          <t>メールサジェスト</t>
-        </is>
-      </c>
-      <c r="D23" s="10" t="inlineStr">
-        <is>
-          <t>emailで「test@」入力</t>
-        </is>
-      </c>
-      <c r="E23" s="10" t="inlineStr">
-        <is>
-          <t>gmail.com等の候補が最大4件表示</t>
-        </is>
-      </c>
-      <c r="F23" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G23" s="10" t="inlineStr"/>
-      <c r="H23" s="10" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="10" t="inlineStr">
-        <is>
-          <t>P5-008</t>
-        </is>
-      </c>
-      <c r="B24" s="10" t="inlineStr">
-        <is>
-          <t>フェーズ5</t>
-        </is>
-      </c>
-      <c r="C24" s="10" t="inlineStr">
-        <is>
-          <t>サジェスト選択</t>
-        </is>
-      </c>
-      <c r="D24" s="10" t="inlineStr">
-        <is>
-          <t>候補をクリック</t>
-        </is>
-      </c>
-      <c r="E24" s="10" t="inlineStr">
-        <is>
-          <t>メールアドレスが補完される</t>
-        </is>
-      </c>
-      <c r="F24" s="10" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G24" s="10" t="inlineStr"/>
-      <c r="H24" s="10" t="inlineStr">
-        <is>
-          <t>2026/04/06</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H118"/>
+  <dimension ref="A1:H141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13948,6 +12996,744 @@
           <t>CSV仕様対応: attachSurnameAlert適用</t>
         </is>
       </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr"/>
+      <c r="B119" t="inlineStr"/>
+      <c r="C119" t="inlineStr"/>
+      <c r="D119" t="inlineStr"/>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="inlineStr"/>
+      <c r="H119" t="inlineStr"/>
+    </row>
+    <row r="120" ht="20" customHeight="1">
+      <c r="A120" s="12" t="inlineStr">
+        <is>
+          <t>【フェーズ2〜5追加】カメラ機能 / QR転送 / OCR自動入力 / 自動補完</t>
+        </is>
+      </c>
+      <c r="B120" s="12" t="inlineStr"/>
+      <c r="C120" s="12" t="inlineStr"/>
+      <c r="D120" s="12" t="inlineStr"/>
+      <c r="E120" s="12" t="inlineStr"/>
+      <c r="F120" s="12" t="inlineStr"/>
+      <c r="G120" s="12" t="inlineStr"/>
+      <c r="H120" s="12" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="13" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="B121" s="13" t="inlineStr">
+        <is>
+          <t>顔写真</t>
+        </is>
+      </c>
+      <c r="C121" s="13" t="inlineStr">
+        <is>
+          <t>カメラモーダル</t>
+        </is>
+      </c>
+      <c r="D121" s="13" t="inlineStr">
+        <is>
+          <t>モーダル表示</t>
+        </is>
+      </c>
+      <c r="E121" s="13" t="inlineStr">
+        <is>
+          <t>スマホで「📷 カメラで撮影」タップ</t>
+        </is>
+      </c>
+      <c r="F121" s="13" t="inlineStr">
+        <is>
+          <t>カメラモーダルが全画面表示・人型ガイドが描画される</t>
+        </is>
+      </c>
+      <c r="G121" s="13" t="n"/>
+      <c r="H121" s="13" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="13" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="B122" s="13" t="inlineStr">
+        <is>
+          <t>顔写真</t>
+        </is>
+      </c>
+      <c r="C122" s="13" t="inlineStr">
+        <is>
+          <t>明るさ判定</t>
+        </is>
+      </c>
+      <c r="D122" s="13" t="inlineStr">
+        <is>
+          <t>暗所判定</t>
+        </is>
+      </c>
+      <c r="E122" s="13" t="inlineStr">
+        <is>
+          <t>暗い場所でカメラを向ける</t>
+        </is>
+      </c>
+      <c r="F122" s="13" t="inlineStr">
+        <is>
+          <t>「明るい場所で撮影してください」が表示される</t>
+        </is>
+      </c>
+      <c r="G122" s="13" t="n"/>
+      <c r="H122" s="13" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="13" t="inlineStr">
+        <is>
+          <t>P03</t>
+        </is>
+      </c>
+      <c r="B123" s="13" t="inlineStr">
+        <is>
+          <t>顔写真</t>
+        </is>
+      </c>
+      <c r="C123" s="13" t="inlineStr">
+        <is>
+          <t>自動シャッター</t>
+        </is>
+      </c>
+      <c r="D123" s="13" t="inlineStr">
+        <is>
+          <t>OFF→ON切替</t>
+        </is>
+      </c>
+      <c r="E123" s="13" t="inlineStr">
+        <is>
+          <t>「🔴 自動 OFF」ボタンをタップ</t>
+        </is>
+      </c>
+      <c r="F123" s="13" t="inlineStr">
+        <is>
+          <t>「🟢 自動 ON」に変わる</t>
+        </is>
+      </c>
+      <c r="G123" s="13" t="n"/>
+      <c r="H123" s="13" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="13" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="B124" s="13" t="inlineStr">
+        <is>
+          <t>顔写真</t>
+        </is>
+      </c>
+      <c r="C124" s="13" t="inlineStr">
+        <is>
+          <t>自動シャッター</t>
+        </is>
+      </c>
+      <c r="D124" s="13" t="inlineStr">
+        <is>
+          <t>自動撮影発火</t>
+        </is>
+      </c>
+      <c r="E124" s="13" t="inlineStr">
+        <is>
+          <t>自動ON・全条件0.5秒クリア</t>
+        </is>
+      </c>
+      <c r="F124" s="13" t="inlineStr">
+        <is>
+          <t>「自動撮影します！」ポップアップ→自動撮影される</t>
+        </is>
+      </c>
+      <c r="G124" s="13" t="n"/>
+      <c r="H124" s="13" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="13" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="B125" s="13" t="inlineStr">
+        <is>
+          <t>顔写真</t>
+        </is>
+      </c>
+      <c r="C125" s="13" t="inlineStr">
+        <is>
+          <t>品質スコア</t>
+        </is>
+      </c>
+      <c r="D125" s="13" t="inlineStr">
+        <is>
+          <t>スコア90以上</t>
+        </is>
+      </c>
+      <c r="E125" s="13" t="inlineStr">
+        <is>
+          <t>明るい・正面・適切サイズで撮影</t>
+        </is>
+      </c>
+      <c r="F125" s="13" t="inlineStr">
+        <is>
+          <t>✅高品質と表示・「この写真を使用する」ボタンが表示</t>
+        </is>
+      </c>
+      <c r="G125" s="13" t="n"/>
+      <c r="H125" s="13" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="13" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="B126" s="13" t="inlineStr">
+        <is>
+          <t>顔写真</t>
+        </is>
+      </c>
+      <c r="C126" s="13" t="inlineStr">
+        <is>
+          <t>品質スコア</t>
+        </is>
+      </c>
+      <c r="D126" s="13" t="inlineStr">
+        <is>
+          <t>スコア60未満</t>
+        </is>
+      </c>
+      <c r="E126" s="13" t="inlineStr">
+        <is>
+          <t>暗い・顔が小さいNG条件で撮影</t>
+        </is>
+      </c>
+      <c r="F126" s="13" t="inlineStr">
+        <is>
+          <t>❌再撮影推奨・「この写真を使用する」ボタンが非表示</t>
+        </is>
+      </c>
+      <c r="G126" s="13" t="n"/>
+      <c r="H126" s="13" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="13" t="inlineStr">
+        <is>
+          <t>P07</t>
+        </is>
+      </c>
+      <c r="B127" s="13" t="inlineStr">
+        <is>
+          <t>顔写真</t>
+        </is>
+      </c>
+      <c r="C127" s="13" t="inlineStr">
+        <is>
+          <t>再撮影</t>
+        </is>
+      </c>
+      <c r="D127" s="13" t="inlineStr">
+        <is>
+          <t>再撮影導線</t>
+        </is>
+      </c>
+      <c r="E127" s="13" t="inlineStr">
+        <is>
+          <t>「再撮影する」をタップ</t>
+        </is>
+      </c>
+      <c r="F127" s="13" t="inlineStr">
+        <is>
+          <t>カメラガイドに戻る</t>
+        </is>
+      </c>
+      <c r="G127" s="13" t="n"/>
+      <c r="H127" s="13" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="13" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="B128" s="13" t="inlineStr">
+        <is>
+          <t>顔写真</t>
+        </is>
+      </c>
+      <c r="C128" s="13" t="inlineStr">
+        <is>
+          <t>QRボタン</t>
+        </is>
+      </c>
+      <c r="D128" s="13" t="inlineStr">
+        <is>
+          <t>PC限定表示</t>
+        </is>
+      </c>
+      <c r="E128" s="13" t="inlineStr">
+        <is>
+          <t>PC表示で顔写真欄を確認</t>
+        </is>
+      </c>
+      <c r="F128" s="13" t="inlineStr">
+        <is>
+          <t>「📱 スマホから送信（QR）」ボタンが表示される</t>
+        </is>
+      </c>
+      <c r="G128" s="13" t="n"/>
+      <c r="H128" s="13" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="13" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="B129" s="13" t="inlineStr">
+        <is>
+          <t>顔写真</t>
+        </is>
+      </c>
+      <c r="C129" s="13" t="inlineStr">
+        <is>
+          <t>QR生成</t>
+        </is>
+      </c>
+      <c r="D129" s="13" t="inlineStr">
+        <is>
+          <t>QRコード表示</t>
+        </is>
+      </c>
+      <c r="E129" s="13" t="inlineStr">
+        <is>
+          <t>「📱 スマホから送信」クリック</t>
+        </is>
+      </c>
+      <c r="F129" s="13" t="inlineStr">
+        <is>
+          <t>QRコードとカウントダウンバーが表示される</t>
+        </is>
+      </c>
+      <c r="G129" s="13" t="n"/>
+      <c r="H129" s="13" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="13" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B130" s="13" t="inlineStr">
+        <is>
+          <t>顔写真</t>
+        </is>
+      </c>
+      <c r="C130" s="13" t="inlineStr">
+        <is>
+          <t>QR転送</t>
+        </is>
+      </c>
+      <c r="D130" s="13" t="inlineStr">
+        <is>
+          <t>SP専用UI表示</t>
+        </is>
+      </c>
+      <c r="E130" s="13" t="inlineStr">
+        <is>
+          <t>QRのURLをスマホで開く</t>
+        </is>
+      </c>
+      <c r="F130" s="13" t="inlineStr">
+        <is>
+          <t>フォーム非表示→「顔写真をPCに送信」専用UIが表示</t>
+        </is>
+      </c>
+      <c r="G130" s="13" t="n"/>
+      <c r="H130" s="13" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="13" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="B131" s="13" t="inlineStr">
+        <is>
+          <t>顔写真</t>
+        </is>
+      </c>
+      <c r="C131" s="13" t="inlineStr">
+        <is>
+          <t>QR転送</t>
+        </is>
+      </c>
+      <c r="D131" s="13" t="inlineStr">
+        <is>
+          <t>タイムアウト</t>
+        </is>
+      </c>
+      <c r="E131" s="13" t="inlineStr">
+        <is>
+          <t>QR表示後5分放置</t>
+        </is>
+      </c>
+      <c r="F131" s="13" t="inlineStr">
+        <is>
+          <t>QRがグレーアウトし「期限切れ」メッセージが表示</t>
+        </is>
+      </c>
+      <c r="G131" s="13" t="n"/>
+      <c r="H131" s="13" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="13" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="B132" s="13" t="inlineStr">
+        <is>
+          <t>顔写真</t>
+        </is>
+      </c>
+      <c r="C132" s="13" t="inlineStr">
+        <is>
+          <t>QR転送</t>
+        </is>
+      </c>
+      <c r="D132" s="13" t="inlineStr">
+        <is>
+          <t>SP→PC転送</t>
+        </is>
+      </c>
+      <c r="E132" s="13" t="inlineStr">
+        <is>
+          <t>SP側で撮影して送信</t>
+        </is>
+      </c>
+      <c r="F132" s="13" t="inlineStr">
+        <is>
+          <t>PC側に写真がプレビュー表示される</t>
+        </is>
+      </c>
+      <c r="G132" s="13" t="n"/>
+      <c r="H132" s="13" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="13" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="B133" s="13" t="inlineStr">
+        <is>
+          <t>顔写真</t>
+        </is>
+      </c>
+      <c r="C133" s="13" t="inlineStr">
+        <is>
+          <t>分析ログ</t>
+        </is>
+      </c>
+      <c r="D133" s="13" t="inlineStr">
+        <is>
+          <t>デバッグパネル</t>
+        </is>
+      </c>
+      <c r="E133" s="13" t="inlineStr">
+        <is>
+          <t>?debug=1でアクセス</t>
+        </is>
+      </c>
+      <c r="F133" s="13" t="inlineStr">
+        <is>
+          <t>撮影統計パネルがページ下部に表示される</t>
+        </is>
+      </c>
+      <c r="G133" s="13" t="n"/>
+      <c r="H133" s="13" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="13" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B134" s="13" t="inlineStr">
+        <is>
+          <t>パスポート</t>
+        </is>
+      </c>
+      <c r="C134" s="13" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="D134" s="13" t="inlineStr">
+        <is>
+          <t>OCR自動起動</t>
+        </is>
+      </c>
+      <c r="E134" s="13" t="inlineStr">
+        <is>
+          <t>パスポート画像をアップロード</t>
+        </is>
+      </c>
+      <c r="F134" s="13" t="inlineStr">
+        <is>
+          <t>処理完了後「🔍 パスポートを読み取り中」が自動表示</t>
+        </is>
+      </c>
+      <c r="G134" s="13" t="n"/>
+      <c r="H134" s="13" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="13" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="B135" s="13" t="inlineStr">
+        <is>
+          <t>パスポート</t>
+        </is>
+      </c>
+      <c r="C135" s="13" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="D135" s="13" t="inlineStr">
+        <is>
+          <t>OCR自動入力</t>
+        </is>
+      </c>
+      <c r="E135" s="13" t="inlineStr">
+        <is>
+          <t>日本パスポートをアップロード</t>
+        </is>
+      </c>
+      <c r="F135" s="13" t="inlineStr">
+        <is>
+          <t>姓・名・パスポート番号・生年月日・有効期限・性別が自動入力</t>
+        </is>
+      </c>
+      <c r="G135" s="13" t="n"/>
+      <c r="H135" s="13" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="13" t="inlineStr">
+        <is>
+          <t>P16</t>
+        </is>
+      </c>
+      <c r="B136" s="13" t="inlineStr">
+        <is>
+          <t>パスポート</t>
+        </is>
+      </c>
+      <c r="C136" s="13" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="D136" s="13" t="inlineStr">
+        <is>
+          <t>OCR失敗</t>
+        </is>
+      </c>
+      <c r="E136" s="13" t="inlineStr">
+        <is>
+          <t>ぼやけた画像をアップロード</t>
+        </is>
+      </c>
+      <c r="F136" s="13" t="inlineStr">
+        <is>
+          <t>「❌ MRZ読取失敗」と「🔄 再読み取り」ボタンが表示</t>
+        </is>
+      </c>
+      <c r="G136" s="13" t="n"/>
+      <c r="H136" s="13" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="13" t="inlineStr">
+        <is>
+          <t>P17</t>
+        </is>
+      </c>
+      <c r="B137" s="13" t="inlineStr">
+        <is>
+          <t>全体</t>
+        </is>
+      </c>
+      <c r="C137" s="13" t="inlineStr">
+        <is>
+          <t>入力履歴</t>
+        </is>
+      </c>
+      <c r="D137" s="13" t="inlineStr">
+        <is>
+          <t>自動保存</t>
+        </is>
+      </c>
+      <c r="E137" s="13" t="inlineStr">
+        <is>
+          <t>Step1入力後Step2へ進む</t>
+        </is>
+      </c>
+      <c r="F137" s="13" t="inlineStr">
+        <is>
+          <t>localStorageにフォームデータが保存される</t>
+        </is>
+      </c>
+      <c r="G137" s="13" t="n"/>
+      <c r="H137" s="13" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="13" t="inlineStr">
+        <is>
+          <t>P18</t>
+        </is>
+      </c>
+      <c r="B138" s="13" t="inlineStr">
+        <is>
+          <t>全体</t>
+        </is>
+      </c>
+      <c r="C138" s="13" t="inlineStr">
+        <is>
+          <t>入力履歴</t>
+        </is>
+      </c>
+      <c r="D138" s="13" t="inlineStr">
+        <is>
+          <t>復元バー表示</t>
+        </is>
+      </c>
+      <c r="E138" s="13" t="inlineStr">
+        <is>
+          <t>保存後にページをリロード</t>
+        </is>
+      </c>
+      <c r="F138" s="13" t="inlineStr">
+        <is>
+          <t>「📋 前回の入力内容があります」バーが表示される</t>
+        </is>
+      </c>
+      <c r="G138" s="13" t="n"/>
+      <c r="H138" s="13" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="13" t="inlineStr">
+        <is>
+          <t>P19</t>
+        </is>
+      </c>
+      <c r="B139" s="13" t="inlineStr">
+        <is>
+          <t>全体</t>
+        </is>
+      </c>
+      <c r="C139" s="13" t="inlineStr">
+        <is>
+          <t>入力履歴</t>
+        </is>
+      </c>
+      <c r="D139" s="13" t="inlineStr">
+        <is>
+          <t>復元実行</t>
+        </is>
+      </c>
+      <c r="E139" s="13" t="inlineStr">
+        <is>
+          <t>「復元する」ボタンをクリック</t>
+        </is>
+      </c>
+      <c r="F139" s="13" t="inlineStr">
+        <is>
+          <t>前回入力した値が各フィールドに復元される</t>
+        </is>
+      </c>
+      <c r="G139" s="13" t="n"/>
+      <c r="H139" s="13" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="13" t="inlineStr">
+        <is>
+          <t>P20</t>
+        </is>
+      </c>
+      <c r="B140" s="13" t="inlineStr">
+        <is>
+          <t>メールアドレス</t>
+        </is>
+      </c>
+      <c r="C140" s="13" t="inlineStr">
+        <is>
+          <t>サジェスト</t>
+        </is>
+      </c>
+      <c r="D140" s="13" t="inlineStr">
+        <is>
+          <t>ドメイン候補</t>
+        </is>
+      </c>
+      <c r="E140" s="13" t="inlineStr">
+        <is>
+          <t>emailフィールドで「test@」を入力</t>
+        </is>
+      </c>
+      <c r="F140" s="13" t="inlineStr">
+        <is>
+          <t>gmail.com等の候補が最大4件表示される</t>
+        </is>
+      </c>
+      <c r="G140" s="13" t="n"/>
+      <c r="H140" s="13" t="n"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="13" t="inlineStr">
+        <is>
+          <t>P21</t>
+        </is>
+      </c>
+      <c r="B141" s="13" t="inlineStr">
+        <is>
+          <t>メールアドレス</t>
+        </is>
+      </c>
+      <c r="C141" s="13" t="inlineStr">
+        <is>
+          <t>サジェスト</t>
+        </is>
+      </c>
+      <c r="D141" s="13" t="inlineStr">
+        <is>
+          <t>サジェスト選択</t>
+        </is>
+      </c>
+      <c r="E141" s="13" t="inlineStr">
+        <is>
+          <t>候補のドメインをクリック</t>
+        </is>
+      </c>
+      <c r="F141" s="13" t="inlineStr">
+        <is>
+          <t>メールアドレスが補完される</t>
+        </is>
+      </c>
+      <c r="G141" s="13" t="n"/>
+      <c r="H141" s="13" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H118"/>

</xml_diff>